<commit_message>
data: weekly EFK refresh (2026-09-15)
</commit_message>
<xml_diff>
--- a/files/exports/de/financings_31_budgetT.xlsx
+++ b/files/exports/de/financings_31_budgetT.xlsx
@@ -354,7 +354,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="30.800000000000004" min="1" max="1" bestFit="1" customWidth="1"/>
@@ -459,7 +459,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3">
-        <v>46248.71739555391</v>
+        <v>46274.64037795565</v>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
@@ -519,7 +519,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3">
-        <v>46248.71739555947</v>
+        <v>46274.64037796136</v>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
@@ -579,7 +579,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3">
-        <v>46248.71739556156</v>
+        <v>46274.64037796367</v>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
@@ -639,7 +639,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3">
-        <v>46248.717395563144</v>
+        <v>46274.640377985954</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
@@ -695,6 +695,66 @@
       </c>
       <c r="P5" s="7" t="n">
         <v>0.0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3">
+        <v>46274.640377989235</v>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Wahrung der schweizerischen Neutralität (Neutralitätsinitiative)</t>
+        </is>
+      </c>
+      <c r="C6" s="5">
+        <v>46292.0</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>329</v>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>MASS-VOLL!</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>607</v>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Annahme der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>1590</v>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung der budgetierten Einnahmen</t>
+        </is>
+      </c>
+      <c r="K6" s="7" t="n">
+        <v>15000.0</v>
+      </c>
+      <c r="L6" s="7" t="n">
+        <v>5800.0</v>
+      </c>
+      <c r="M6" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N6" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="O6" s="7" t="n">
+        <v>2800.0</v>
+      </c>
+      <c r="P6" s="7" t="n">
+        <v>6400.0</v>
       </c>
     </row>
   </sheetData>
@@ -852,7 +912,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3">
-        <v>46248.71739556598</v>
+        <v>46274.64037799259</v>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
@@ -932,7 +992,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3">
-        <v>46248.71739556835</v>
+        <v>46274.64037799534</v>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
@@ -1004,7 +1064,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3">
-        <v>46248.717395569685</v>
+        <v>46274.64037799703</v>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
@@ -1076,7 +1136,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3">
-        <v>46248.717395571286</v>
+        <v>46274.640377998454</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
@@ -1148,7 +1208,7 @@
     </row>
     <row r="6">
       <c r="A6" s="3">
-        <v>46248.71739557247</v>
+        <v>46274.64037799983</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
@@ -1220,7 +1280,7 @@
     </row>
     <row r="7">
       <c r="A7" s="3">
-        <v>46248.717395573556</v>
+        <v>46274.6403780012</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
@@ -1300,7 +1360,7 @@
     </row>
     <row r="8">
       <c r="A8" s="3">
-        <v>46248.717395574684</v>
+        <v>46274.64037800282</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
@@ -1372,7 +1432,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3">
-        <v>46248.71739557574</v>
+        <v>46274.64037800416</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
data: weekly EFK refresh (2026-09-19)
</commit_message>
<xml_diff>
--- a/files/exports/de/financings_31_budgetT.xlsx
+++ b/files/exports/de/financings_31_budgetT.xlsx
@@ -354,7 +354,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P6"/>
+  <dimension ref="A1:P7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="30.800000000000004" min="1" max="1" bestFit="1" customWidth="1"/>
@@ -459,7 +459,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3">
-        <v>46274.64037795565</v>
+        <v>46282.425430499534</v>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
@@ -519,7 +519,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3">
-        <v>46274.64037796136</v>
+        <v>46282.42543050405</v>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
@@ -559,10 +559,10 @@
         </is>
       </c>
       <c r="K3" s="7" t="n">
-        <v>3842800.0</v>
+        <v>5691982.0</v>
       </c>
       <c r="L3" s="7" t="n">
-        <v>3842800.0</v>
+        <v>5691982.0</v>
       </c>
       <c r="M3" s="7" t="n">
         <v>0.0</v>
@@ -579,7 +579,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3">
-        <v>46274.64037796367</v>
+        <v>46282.425430505704</v>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
@@ -619,10 +619,10 @@
         </is>
       </c>
       <c r="K4" s="7" t="n">
-        <v>366830.0</v>
+        <v>520830.0</v>
       </c>
       <c r="L4" s="7" t="n">
-        <v>361000.0</v>
+        <v>515000.0</v>
       </c>
       <c r="M4" s="7" t="n">
         <v>0.0</v>
@@ -639,7 +639,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3">
-        <v>46274.640377985954</v>
+        <v>46282.42543050706</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
@@ -699,7 +699,7 @@
     </row>
     <row r="6">
       <c r="A6" s="3">
-        <v>46274.640377989235</v>
+        <v>46282.425430508534</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
@@ -755,6 +755,66 @@
       </c>
       <c r="P6" s="7" t="n">
         <v>6400.0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3">
+        <v>46282.42543050989</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Wahrung der schweizerischen Neutralität (Neutralitätsinitiative)</t>
+        </is>
+      </c>
+      <c r="C7" s="5">
+        <v>46292.0</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>457</v>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Junge Schweizerische Volkspartei</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>608</v>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Annahme der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>1591</v>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung der budgetierten Einnahmen</t>
+        </is>
+      </c>
+      <c r="K7" s="7" t="n">
+        <v>51263.95</v>
+      </c>
+      <c r="L7" s="7" t="n">
+        <v>42000.0</v>
+      </c>
+      <c r="M7" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N7" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="O7" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="P7" s="7" t="n">
+        <v>9263.95</v>
       </c>
     </row>
   </sheetData>
@@ -771,7 +831,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:V9"/>
+  <dimension ref="A1:V11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="30.800000000000004" min="1" max="1" bestFit="1" customWidth="1"/>
@@ -912,7 +972,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3">
-        <v>46274.64037799259</v>
+        <v>46282.425430512194</v>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
@@ -952,7 +1012,7 @@
         </is>
       </c>
       <c r="K2" s="6" t="n">
-        <v>4592</v>
+        <v>4610</v>
       </c>
       <c r="L2" s="4" t="inlineStr">
         <is>
@@ -992,7 +1052,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3">
-        <v>46274.64037799534</v>
+        <v>46282.42543051434</v>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
@@ -1032,7 +1092,7 @@
         </is>
       </c>
       <c r="K3" s="6" t="n">
-        <v>4593</v>
+        <v>4611</v>
       </c>
       <c r="L3" s="4"/>
       <c r="M3" s="4"/>
@@ -1064,7 +1124,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3">
-        <v>46274.64037799703</v>
+        <v>46282.42543051557</v>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
@@ -1104,7 +1164,7 @@
         </is>
       </c>
       <c r="K4" s="6" t="n">
-        <v>4594</v>
+        <v>4612</v>
       </c>
       <c r="L4" s="4"/>
       <c r="M4" s="4"/>
@@ -1136,7 +1196,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3">
-        <v>46274.640377998454</v>
+        <v>46282.42543051661</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
@@ -1176,7 +1236,7 @@
         </is>
       </c>
       <c r="K5" s="6" t="n">
-        <v>4595</v>
+        <v>4613</v>
       </c>
       <c r="L5" s="4"/>
       <c r="M5" s="4"/>
@@ -1208,7 +1268,7 @@
     </row>
     <row r="6">
       <c r="A6" s="3">
-        <v>46274.64037799983</v>
+        <v>46282.425430517615</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
@@ -1248,7 +1308,7 @@
         </is>
       </c>
       <c r="K6" s="6" t="n">
-        <v>4596</v>
+        <v>4614</v>
       </c>
       <c r="L6" s="4"/>
       <c r="M6" s="4"/>
@@ -1280,7 +1340,7 @@
     </row>
     <row r="7">
       <c r="A7" s="3">
-        <v>46274.6403780012</v>
+        <v>46282.42543051863</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
@@ -1320,7 +1380,7 @@
         </is>
       </c>
       <c r="K7" s="6" t="n">
-        <v>4597</v>
+        <v>4615</v>
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
@@ -1360,7 +1420,7 @@
     </row>
     <row r="8">
       <c r="A8" s="3">
-        <v>46274.64037800282</v>
+        <v>46282.42543051969</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
@@ -1400,7 +1460,7 @@
         </is>
       </c>
       <c r="K8" s="6" t="n">
-        <v>4598</v>
+        <v>4616</v>
       </c>
       <c r="L8" s="4"/>
       <c r="M8" s="4"/>
@@ -1432,7 +1492,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3">
-        <v>46274.64037800416</v>
+        <v>46282.425430520714</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
@@ -1443,11 +1503,11 @@
         <v>46292.0</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Überparteiliches Komitee Nein zur Neutralitätsinitiative</t>
+          <t>Wahrung der Schweizer Neutralität</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -1456,15 +1516,15 @@
         </is>
       </c>
       <c r="G9" s="6" t="n">
-        <v>605</v>
+        <v>602</v>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Ablehnung der Abstimmungsvorlage</t>
+          <t>Annahme der Abstimmungsvorlage</t>
         </is>
       </c>
       <c r="I9" s="6" t="n">
-        <v>1574</v>
+        <v>1580</v>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
@@ -1472,22 +1532,30 @@
         </is>
       </c>
       <c r="K9" s="6" t="n">
-        <v>4566</v>
-      </c>
-      <c r="L9" s="4"/>
-      <c r="M9" s="4"/>
-      <c r="N9" s="4"/>
-      <c r="O9" s="4"/>
-      <c r="P9" s="4" t="inlineStr">
-        <is>
-          <t>economiesuisse Verband der Schweizer Unternehmen</t>
-        </is>
-      </c>
-      <c r="Q9" s="4" t="inlineStr">
-        <is>
-          <t>Zürich</t>
-        </is>
-      </c>
+        <v>4617</v>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>Blocher</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="inlineStr">
+        <is>
+          <t>Christoph</t>
+        </is>
+      </c>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t>Herrliberg</t>
+        </is>
+      </c>
+      <c r="O9" s="4" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="P9" s="4"/>
+      <c r="Q9" s="4"/>
       <c r="R9" s="4" t="inlineStr">
         <is>
           <t>Monetär</t>
@@ -1496,9 +1564,161 @@
       <c r="S9" s="4"/>
       <c r="T9" s="4"/>
       <c r="U9" s="7" t="n">
+        <v>1000000.0</v>
+      </c>
+      <c r="V9" s="5">
+        <v>46280.0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3">
+        <v>46282.4254305219</v>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Wahrung der schweizerischen Neutralität (Neutralitätsinitiative)</t>
+        </is>
+      </c>
+      <c r="C10" s="5">
+        <v>46292.0</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>460</v>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Wahrung der Schweizer Neutralität</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>602</v>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Annahme der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>1580</v>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung von Zuwendungen über 15 000 Franken</t>
+        </is>
+      </c>
+      <c r="K10" s="6" t="n">
+        <v>4618</v>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>Blocher</t>
+        </is>
+      </c>
+      <c r="M10" s="4" t="inlineStr">
+        <is>
+          <t>Christoph</t>
+        </is>
+      </c>
+      <c r="N10" s="4" t="inlineStr">
+        <is>
+          <t>Herrliberg</t>
+        </is>
+      </c>
+      <c r="O10" s="4" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="P10" s="4"/>
+      <c r="Q10" s="4"/>
+      <c r="R10" s="4" t="inlineStr">
+        <is>
+          <t>Monetär</t>
+        </is>
+      </c>
+      <c r="S10" s="4"/>
+      <c r="T10" s="4"/>
+      <c r="U10" s="7" t="n">
+        <v>850000.0</v>
+      </c>
+      <c r="V10" s="5">
+        <v>46280.0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3">
+        <v>46282.425430522955</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Wahrung der schweizerischen Neutralität (Neutralitätsinitiative)</t>
+        </is>
+      </c>
+      <c r="C11" s="5">
+        <v>46292.0</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>459</v>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Überparteiliches Komitee Nein zur Neutralitätsinitiative</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>605</v>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Ablehnung der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>1574</v>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung von Zuwendungen über 15 000 Franken</t>
+        </is>
+      </c>
+      <c r="K11" s="6" t="n">
+        <v>4566</v>
+      </c>
+      <c r="L11" s="4"/>
+      <c r="M11" s="4"/>
+      <c r="N11" s="4"/>
+      <c r="O11" s="4"/>
+      <c r="P11" s="4" t="inlineStr">
+        <is>
+          <t>economiesuisse Verband der Schweizer Unternehmen</t>
+        </is>
+      </c>
+      <c r="Q11" s="4" t="inlineStr">
+        <is>
+          <t>Zürich</t>
+        </is>
+      </c>
+      <c r="R11" s="4" t="inlineStr">
+        <is>
+          <t>Monetär</t>
+        </is>
+      </c>
+      <c r="S11" s="4"/>
+      <c r="T11" s="4"/>
+      <c r="U11" s="7" t="n">
         <v>1200000.0</v>
       </c>
-      <c r="V9" s="5">
+      <c r="V11" s="5">
         <v>46162.0</v>
       </c>
     </row>

</xml_diff>